<commit_message>
hoan thien challenge 2
</commit_message>
<xml_diff>
--- a/Chalenge2/reports/modeling.xlsx
+++ b/Chalenge2/reports/modeling.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ml_personalNGroup\Group\chalenge2\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E58FD5AD-909A-49C3-AD97-B319D539FC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C33F3A-E38D-4E15-BF71-6DD857C448C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="2530" windowWidth="19200" windowHeight="9350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Thời gian chạy</t>
   </si>
@@ -31,13 +31,22 @@
     <t>Kết luận</t>
   </si>
   <si>
-    <t>2025-10-27 21:01:28</t>
+    <t>2025-10-31 08:59:02</t>
+  </si>
+  <si>
+    <t>Chia dữ liệu train/validation 80/20 cho mô hình XGBoost</t>
   </si>
   <si>
     <t>Dữ liệu đã được chia hợp lý giúp đánh giá mô hình khách quan, tránh overfitting</t>
   </si>
   <si>
-    <t>Chia dữ liệu train/validation 80/20</t>
+    <t>2025-10-31 08:59:31</t>
+  </si>
+  <si>
+    <t>Tính RMSE cho Ridge Regression</t>
+  </si>
+  <si>
+    <t>RMSE Ridge = 0.13902</t>
   </si>
 </sst>
 </file>
@@ -400,11 +409,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.1796875" customWidth="1"/>
-    <col min="2" max="2" width="75.08984375" customWidth="1"/>
+    <col min="1" max="1" width="32.08984375" customWidth="1"/>
+    <col min="2" max="2" width="95.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -423,10 +432,21 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>4</v>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
minh chung excel cho modeling
</commit_message>
<xml_diff>
--- a/Chalenge2/reports/modeling.xlsx
+++ b/Chalenge2/reports/modeling.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ml_personalNGroup\Group\chalenge2\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C33F3A-E38D-4E15-BF71-6DD857C448C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F11A97-F9AD-4146-8E36-99561F1C4056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="2530" windowWidth="19200" windowHeight="9350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>Thời gian chạy</t>
   </si>
@@ -47,6 +47,63 @@
   </si>
   <si>
     <t>RMSE Ridge = 0.13902</t>
+  </si>
+  <si>
+    <t>2025-10-31 09:22:17</t>
+  </si>
+  <si>
+    <t>Huấn luyện và đánh giá Ridge</t>
+  </si>
+  <si>
+    <t>2025-10-31 09:22:23</t>
+  </si>
+  <si>
+    <t>Huấn luyện và đánh giá RandomForest</t>
+  </si>
+  <si>
+    <t>RMSE RandomForest = 0.14756</t>
+  </si>
+  <si>
+    <t>2025-10-31 09:22:25</t>
+  </si>
+  <si>
+    <t>Huấn luyện và đánh giá XGBoost</t>
+  </si>
+  <si>
+    <t>RMSE XGBoost = 0.13902</t>
+  </si>
+  <si>
+    <t>Huấn luyện và đánh giá LightGBM</t>
+  </si>
+  <si>
+    <t>RMSE LightGBM = 0.13857</t>
+  </si>
+  <si>
+    <t>2025-10-31 09:25:00</t>
+  </si>
+  <si>
+    <t>Optuna tìm siêu tham số tối ưu cho XGBoost</t>
+  </si>
+  <si>
+    <t>Best params: {'n_estimators': 412, 'learning_rate': 0.03311345167435121, 'max_depth': 4, 'subsample': 0.8414736058154724, 'colsample_bytree': 0.9136397871275272, 'gamma': 0.0010197380486226277, 'min_child_weight': 1}, Best RMSE (CV): 0.12367</t>
+  </si>
+  <si>
+    <t>2025-10-31 09:26:58</t>
+  </si>
+  <si>
+    <t>Huấn luyện mô hình XGBoost với best_params trên toàn bộ dữ liệu</t>
+  </si>
+  <si>
+    <t>Đã huấn luyện xong, mô hình sẵn sàng sử dụng</t>
+  </si>
+  <si>
+    <t>2025-10-31 09:30:21</t>
+  </si>
+  <si>
+    <t>Đánh giá hiệu suất mô hình XGBoost trên train/validation</t>
+  </si>
+  <si>
+    <t>RMSE Train: 0.03164, RMSE Validation: 0.03301, R² Train: 0.9934, R² Validation: 0.9942</t>
   </si>
 </sst>
 </file>
@@ -409,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32.08984375" customWidth="1"/>
@@ -449,6 +506,83 @@
         <v>8</v>
       </c>
     </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>